<commit_message>
Remove studiekeuzeprofiel and integrate 1cho data
</commit_message>
<xml_diff>
--- a/R/data/1cho/variabelen.xlsx
+++ b/R/data/1cho/variabelen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahtanjung/Projects/LTA_lta-hhs-fairnessawareness/R/data/1cho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2B92B36D-F572-134A-B81B-5CC0CE2C794B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{18063DB7-F7DF-554D-8BEE-7E05D01CE5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14540" yWindow="680" windowWidth="20700" windowHeight="17760" xr2:uid="{C23F249F-BD44-6E44-9A12-289A2EF10B11}"/>
   </bookViews>
@@ -882,9 +882,6 @@
     <t>aansluiting</t>
   </si>
   <si>
-    <t>ID</t>
-  </si>
-  <si>
     <t>INS_Collegejaar</t>
   </si>
   <si>
@@ -934,6 +931,9 @@
   </si>
   <si>
     <t>SUC_Retentie</t>
+  </si>
+  <si>
+    <t>INS_Student_UUID_opleiding_vorm</t>
   </si>
 </sst>
 </file>
@@ -1847,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>285</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -2458,7 +2458,7 @@
         <v>1</v>
       </c>
       <c r="D57" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -2472,7 +2472,7 @@
         <v>0</v>
       </c>
       <c r="D58" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -3124,7 +3124,7 @@
         <v>0</v>
       </c>
       <c r="D117" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
@@ -3138,7 +3138,7 @@
         <v>0</v>
       </c>
       <c r="D118" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
@@ -3207,7 +3207,7 @@
         <v>0</v>
       </c>
       <c r="D124" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
@@ -3254,7 +3254,7 @@
         <v>0</v>
       </c>
       <c r="D128" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="D129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
@@ -4767,7 +4767,7 @@
         <v>0</v>
       </c>
       <c r="D265" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.2">
@@ -4792,7 +4792,7 @@
         <v>0</v>
       </c>
       <c r="D267" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.2">
@@ -4806,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="D268" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.2">
@@ -4820,7 +4820,7 @@
         <v>0</v>
       </c>
       <c r="D269" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.2">
@@ -4834,7 +4834,7 @@
         <v>0</v>
       </c>
       <c r="D270" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.2">
@@ -4848,7 +4848,7 @@
         <v>0</v>
       </c>
       <c r="D271" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.2">
@@ -4918,7 +4918,7 @@
         <v>0</v>
       </c>
       <c r="D276" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.2">
@@ -4932,7 +4932,7 @@
         <v>1</v>
       </c>
       <c r="D277" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.2">
@@ -4946,7 +4946,7 @@
         <v>1</v>
       </c>
       <c r="D278" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>